<commit_message>
Update benchmark: 2026-08-24 06:58:05 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -744,11 +740,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -901,11 +893,7 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -916,11 +904,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -933,11 +917,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -950,21 +930,13 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -977,11 +949,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -1008,11 +976,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-08-25 06:46:44 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -740,7 +744,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -893,7 +901,11 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -904,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -917,12 +933,12 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -930,13 +946,21 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -949,17 +973,13 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -976,7 +996,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-08-26 06:49:41 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -938,7 +938,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -978,8 +982,16 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-28 18:16:54 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -898,14 +894,10 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+          <t>WU: 0,1 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +925,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -977,11 +965,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-29 12:24:13 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -897,7 +901,11 @@
           <t>WU: 0,1 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -925,7 +933,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -965,7 +977,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-30 11:22:30 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,11 +718,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -744,11 +740,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -896,11 +888,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 0,1 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -928,11 +916,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -950,11 +934,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -972,11 +952,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-08-31 12:51:33 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,7 +718,11 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -740,7 +744,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -888,7 +896,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -916,7 +928,11 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -934,7 +950,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -952,7 +972,11 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-02 10:45:49 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -901,11 +901,7 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +929,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -945,11 +937,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -977,11 +965,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -997,11 +981,7 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-03 10:46:32 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -901,7 +897,11 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -912,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -929,7 +925,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -937,7 +937,11 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -948,11 +952,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -965,7 +965,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -981,18 +985,18 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-09-04 10:43:54 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -952,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -996,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-09-05 10:02:50 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -636,11 +636,7 @@
           <t>18 TL - 18 TL</t>
         </is>
       </c>
-      <c r="J2" s="14" t="inlineStr">
-        <is>
-          <t>65 TL - 65 TL</t>
-        </is>
-      </c>
+      <c r="J2" s="14" t="inlineStr"/>
       <c r="K2" s="14" t="inlineStr">
         <is>
           <t>32,62 TL - 32,62 TL</t>
@@ -789,11 +785,7 @@
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr"/>
-      <c r="J7" s="14" t="inlineStr">
-        <is>
-          <t>%3,5</t>
-        </is>
-      </c>
+      <c r="J7" s="14" t="inlineStr"/>
       <c r="K7" s="14" t="inlineStr">
         <is>
           <t>%3,1</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-06 10:22:32 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -636,7 +636,11 @@
           <t>18 TL - 18 TL</t>
         </is>
       </c>
-      <c r="J2" s="14" t="inlineStr"/>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>65 TL - 65 TL</t>
+        </is>
+      </c>
       <c r="K2" s="14" t="inlineStr">
         <is>
           <t>32,62 TL - 32,62 TL</t>
@@ -750,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -785,7 +785,11 @@
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr"/>
-      <c r="J7" s="14" t="inlineStr"/>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>%3,5</t>
+        </is>
+      </c>
       <c r="K7" s="14" t="inlineStr">
         <is>
           <t>%3,1</t>
@@ -908,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -952,11 +952,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1000,11 +996,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-09-07 11:44:16 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -952,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -996,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-09-09 10:51:34 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -739,11 +739,7 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="H6" s="14" t="inlineStr"/>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -901,11 +897,7 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +925,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -945,11 +933,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -977,11 +961,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -997,11 +977,7 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-10 10:45:02 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -739,7 +739,11 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -894,7 +898,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr"/>
@@ -908,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -933,7 +933,11 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -944,11 +948,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -977,18 +977,18 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-09-11 10:43:32 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -901,7 +901,11 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -925,7 +933,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -933,22 +945,22 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -961,7 +973,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -977,18 +993,18 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-09-12 10:12:35 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,11 +718,7 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -896,11 +892,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -928,11 +920,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -945,7 +933,11 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -968,11 +960,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
@@ -993,7 +981,11 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-13 11:12:25 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -631,21 +631,9 @@
           <t>15 TL - 15 TL</t>
         </is>
       </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>18 TL - 18 TL</t>
-        </is>
-      </c>
-      <c r="J2" s="14" t="inlineStr">
-        <is>
-          <t>65 TL - 65 TL</t>
-        </is>
-      </c>
-      <c r="K2" s="14" t="inlineStr">
-        <is>
-          <t>32,62 TL - 32,62 TL</t>
-        </is>
-      </c>
+      <c r="I2" s="14" t="inlineStr"/>
+      <c r="J2" s="14" t="inlineStr"/>
+      <c r="K2" s="14" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -718,7 +706,11 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -732,29 +724,17 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
+          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -785,16 +765,8 @@
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr"/>
-      <c r="J7" s="14" t="inlineStr">
-        <is>
-          <t>%3,5</t>
-        </is>
-      </c>
-      <c r="K7" s="14" t="inlineStr">
-        <is>
-          <t>%3,1</t>
-        </is>
-      </c>
+      <c r="J7" s="14" t="inlineStr"/>
+      <c r="K7" s="14" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -811,11 +783,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -831,11 +799,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -851,11 +815,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -871,11 +831,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -892,7 +848,11 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
           <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
@@ -900,19 +860,11 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -920,7 +872,11 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -933,26 +889,10 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -960,7 +900,11 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>
@@ -976,27 +920,11 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="G14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1041,17 +969,17 @@
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar: 220 TL Azami Tutar: 220 TL / 220 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 375 TL Azami Tutar: 375 TL / 6.500 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t>%0,3 Asgari Tutar: 237,26 TL Azami Tutar: 237,26 TL / 298,96 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
     </row>
@@ -1109,17 +1037,17 @@
       </c>
       <c r="I17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar: 220 TL Azami Tutar: </t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 350 TL Azami Tutar: 350 TL / 5.500 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>%0,6 Asgari Tutar: 237,26 TL Azami Tutar: 237,26 TL / 3.034,67 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
     </row>
@@ -1187,21 +1115,9 @@
           <t>100 TL</t>
         </is>
       </c>
-      <c r="I20" s="14" t="inlineStr">
-        <is>
-          <t>30 TL</t>
-        </is>
-      </c>
-      <c r="J20" s="14" t="inlineStr">
-        <is>
-          <t>200 TL</t>
-        </is>
-      </c>
-      <c r="K20" s="14" t="inlineStr">
-        <is>
-          <t>147,11 TL</t>
-        </is>
-      </c>
+      <c r="I20" s="14" t="inlineStr"/>
+      <c r="J20" s="14" t="inlineStr"/>
+      <c r="K20" s="14" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" s="13" t="inlineStr">
@@ -1241,17 +1157,17 @@
       </c>
       <c r="I21" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 240 TL Azami Tutar: 240 TL / 2.325 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 500 TL Azami Tutar: 500 TL / 5.000 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>%0,9 Asgari Tutar: 446,06 TL Azami Tutar: 446,06 TL / 2.427,26 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
     </row>
@@ -1293,17 +1209,17 @@
       </c>
       <c r="I22" s="14" t="inlineStr">
         <is>
-          <t>%0,32 Asgari Tutar: 300 TL Azami Tutar: 300 TL / 300 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 1.500 TL Azami Tutar: 1.500 TL / 9.000 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>%0,3 Asgari Tutar: 73,56 TL Azami Tutar: 73,56 TL / 9.115,86 TL</t>
+          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
         </is>
       </c>
     </row>
@@ -1343,21 +1259,9 @@
           <t>57,5 TL</t>
         </is>
       </c>
-      <c r="I23" s="14" t="inlineStr">
-        <is>
-          <t>455 TL</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="inlineStr">
-        <is>
-          <t>75 TL</t>
-        </is>
-      </c>
-      <c r="K23" s="14" t="inlineStr">
-        <is>
-          <t>64,8 TL</t>
-        </is>
-      </c>
+      <c r="I23" s="14" t="inlineStr"/>
+      <c r="J23" s="14" t="inlineStr"/>
+      <c r="K23" s="14" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
@@ -1390,31 +1294,15 @@
           <t>600 TL</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>160 TL</t>
-        </is>
-      </c>
+      <c r="G24" s="14" t="inlineStr"/>
       <c r="H24" s="14" t="inlineStr">
         <is>
           <t>350 TL</t>
         </is>
       </c>
-      <c r="I24" s="14" t="inlineStr">
-        <is>
-          <t>20 TL</t>
-        </is>
-      </c>
-      <c r="J24" s="14" t="inlineStr">
-        <is>
-          <t>500 TL</t>
-        </is>
-      </c>
-      <c r="K24" s="14" t="inlineStr">
-        <is>
-          <t>446,06 TL</t>
-        </is>
-      </c>
+      <c r="I24" s="14" t="inlineStr"/>
+      <c r="J24" s="14" t="inlineStr"/>
+      <c r="K24" s="14" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="B25" s="13" t="inlineStr">
@@ -1448,21 +1336,9 @@
           <t>400 TL</t>
         </is>
       </c>
-      <c r="I25" s="14" t="inlineStr">
-        <is>
-          <t>300 TL</t>
-        </is>
-      </c>
-      <c r="J25" s="14" t="inlineStr">
-        <is>
-          <t>750 TL</t>
-        </is>
-      </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>374,4 TL</t>
-        </is>
-      </c>
+      <c r="I25" s="14" t="inlineStr"/>
+      <c r="J25" s="14" t="inlineStr"/>
+      <c r="K25" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
Update benchmark: 2026-09-14 11:57:56 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -631,9 +631,21 @@
           <t>15 TL - 15 TL</t>
         </is>
       </c>
-      <c r="I2" s="14" t="inlineStr"/>
-      <c r="J2" s="14" t="inlineStr"/>
-      <c r="K2" s="14" t="inlineStr"/>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>18 TL - 18 TL</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>65 TL - 65 TL</t>
+        </is>
+      </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>32,62 TL - 32,62 TL</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -724,17 +736,29 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr"/>
-      <c r="I6" s="14" t="inlineStr"/>
+          <t>8.300,01 TL - 99,71 TL</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -765,8 +789,16 @@
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr"/>
-      <c r="J7" s="14" t="inlineStr"/>
-      <c r="K7" s="14" t="inlineStr"/>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>%3,5</t>
+        </is>
+      </c>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>%3,1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -783,7 +815,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -799,7 +835,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -815,7 +855,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -831,7 +875,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -860,11 +908,19 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -889,10 +945,26 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
-      <c r="I13" s="14" t="inlineStr"/>
-      <c r="J13" s="14" t="inlineStr"/>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -915,16 +987,28 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
-      <c r="G14" s="14" t="inlineStr"/>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -969,17 +1053,17 @@
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t xml:space="preserve"> Asgari Tutar: 220 TL Azami Tutar: 220 TL / 220 TL</t>
         </is>
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,5 Asgari Tutar: 375 TL Azami Tutar: 375 TL / 6.500 TL</t>
         </is>
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,3 Asgari Tutar: 237,26 TL Azami Tutar: 237,26 TL / 298,96 TL</t>
         </is>
       </c>
     </row>
@@ -1037,17 +1121,17 @@
       </c>
       <c r="I17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t xml:space="preserve"> Asgari Tutar: 220 TL Azami Tutar: </t>
         </is>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,5 Asgari Tutar: 350 TL Azami Tutar: 350 TL / 5.500 TL</t>
         </is>
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,6 Asgari Tutar: 237,26 TL Azami Tutar: 237,26 TL / 3.034,67 TL</t>
         </is>
       </c>
     </row>
@@ -1115,9 +1199,21 @@
           <t>100 TL</t>
         </is>
       </c>
-      <c r="I20" s="14" t="inlineStr"/>
-      <c r="J20" s="14" t="inlineStr"/>
-      <c r="K20" s="14" t="inlineStr"/>
+      <c r="I20" s="14" t="inlineStr">
+        <is>
+          <t>30 TL</t>
+        </is>
+      </c>
+      <c r="J20" s="14" t="inlineStr">
+        <is>
+          <t>200 TL</t>
+        </is>
+      </c>
+      <c r="K20" s="14" t="inlineStr">
+        <is>
+          <t>147,11 TL</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="13" t="inlineStr">
@@ -1157,17 +1253,17 @@
       </c>
       <c r="I21" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,5 Asgari Tutar: 240 TL Azami Tutar: 240 TL / 2.325 TL</t>
         </is>
       </c>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,5 Asgari Tutar: 500 TL Azami Tutar: 500 TL / 5.000 TL</t>
         </is>
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,9 Asgari Tutar: 446,06 TL Azami Tutar: 446,06 TL / 2.427,26 TL</t>
         </is>
       </c>
     </row>
@@ -1209,17 +1305,17 @@
       </c>
       <c r="I22" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,32 Asgari Tutar: 300 TL Azami Tutar: 300 TL / 300 TL</t>
         </is>
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,5 Asgari Tutar: 1.500 TL Azami Tutar: 1.500 TL / 9.000 TL</t>
         </is>
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Asgari Tutar:  Azami Tutar: </t>
+          <t>%0,3 Asgari Tutar: 73,56 TL Azami Tutar: 73,56 TL / 9.115,86 TL</t>
         </is>
       </c>
     </row>
@@ -1259,9 +1355,21 @@
           <t>57,5 TL</t>
         </is>
       </c>
-      <c r="I23" s="14" t="inlineStr"/>
-      <c r="J23" s="14" t="inlineStr"/>
-      <c r="K23" s="14" t="inlineStr"/>
+      <c r="I23" s="14" t="inlineStr">
+        <is>
+          <t>455 TL</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="inlineStr">
+        <is>
+          <t>75 TL</t>
+        </is>
+      </c>
+      <c r="K23" s="14" t="inlineStr">
+        <is>
+          <t>64,8 TL</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
@@ -1294,15 +1402,31 @@
           <t>600 TL</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr"/>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>160 TL</t>
+        </is>
+      </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
           <t>350 TL</t>
         </is>
       </c>
-      <c r="I24" s="14" t="inlineStr"/>
-      <c r="J24" s="14" t="inlineStr"/>
-      <c r="K24" s="14" t="inlineStr"/>
+      <c r="I24" s="14" t="inlineStr">
+        <is>
+          <t>20 TL</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="inlineStr">
+        <is>
+          <t>500 TL</t>
+        </is>
+      </c>
+      <c r="K24" s="14" t="inlineStr">
+        <is>
+          <t>446,06 TL</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="13" t="inlineStr">
@@ -1336,9 +1460,21 @@
           <t>400 TL</t>
         </is>
       </c>
-      <c r="I25" s="14" t="inlineStr"/>
-      <c r="J25" s="14" t="inlineStr"/>
-      <c r="K25" s="14" t="inlineStr"/>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>300 TL</t>
+        </is>
+      </c>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>750 TL</t>
+        </is>
+      </c>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>374,4 TL</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
Update benchmark: 2026-09-15 11:12:52 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -987,7 +987,11 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-17 11:05:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -896,14 +896,10 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+          <t>WU: 6 USD–; Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
@@ -928,11 +924,7 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -972,11 +964,7 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-18 10:41:07 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -896,10 +896,14 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>WU: 6 USD–; Diğer: 700 TL–4.000 TL</t>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr"/>
@@ -924,7 +928,11 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
@@ -964,7 +972,11 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
           <t>3.500 TL - 13.500 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-20 10:44:53 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -916,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -960,11 +952,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1008,11 +996,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-09-21 12:08:44 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -952,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -996,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-09-22 11:04:09 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -987,11 +987,7 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-23 10:54:44 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -631,11 +631,7 @@
           <t>15 TL - 15 TL</t>
         </is>
       </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>18 TL - 18 TL</t>
-        </is>
-      </c>
+      <c r="I2" s="14" t="inlineStr"/>
       <c r="J2" s="14" t="inlineStr">
         <is>
           <t>65 TL - 65 TL</t>
@@ -987,7 +983,11 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-24 11:13:33 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -631,7 +631,11 @@
           <t>15 TL - 15 TL</t>
         </is>
       </c>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>18 TL - 18 TL</t>
+        </is>
+      </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
           <t>65 TL - 65 TL</t>
@@ -936,7 +940,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-25 11:17:34 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -940,7 +940,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -962,7 +962,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 50 TL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-27 11:31:16 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -938,11 +938,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -982,11 +978,7 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-28 13:03:51 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -938,7 +938,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -978,7 +982,11 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-09-30 12:01:32 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -916,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -950,21 +942,13 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -987,11 +971,7 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -1008,11 +988,7 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-01 12:33:42 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -942,13 +950,21 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -971,7 +987,11 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -988,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-04 11:52:28 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -987,11 +987,7 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-06 12:51:46 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -728,11 +728,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -938,11 +934,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -982,11 +974,7 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-07 12:45:39 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -728,28 +728,20 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -897,11 +889,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -912,11 +900,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -929,34 +913,14 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -969,34 +933,22 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1016,7 +968,7 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>%0,8 Asgari Tutar: 285,72 TL Azami Tutar: 285,72 TL / 3.047,62 TL</t>
+          <t>%0,8 Asgari Tutar: 380,95 TL Azami Tutar: 380,95 TL / 4.000 TL</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -1084,7 +1036,7 @@
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>%0,8 Asgari Tutar: 285,72 TL Azami Tutar: 285,72 TL / 3.047,62 TL</t>
+          <t>%0,8 Asgari Tutar: 380,95 TL Azami Tutar: 380,95 TL / 4.000 TL</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
@@ -1168,7 +1120,7 @@
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>285,72 TL</t>
+          <t>380,95 TL</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
@@ -1216,7 +1168,7 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>%0,5 Asgari Tutar: 428,58 TL Azami Tutar: 428,58 TL / 5.523,81 TL</t>
+          <t>%0,5 Asgari Tutar: 761,9 TL Azami Tutar: 761,9 TL / 7.619,04 TL</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -1268,7 +1220,7 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>%1 Asgari Tutar: 285,72 TL Azami Tutar: 285,72 TL / 6.857,15 TL</t>
+          <t>%0,5 Asgari Tutar: 571,43 TL Azami Tutar: 571,43 TL / 12.952,38 TL</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
@@ -1320,7 +1272,7 @@
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>64,77 TL</t>
+          <t>95,24 TL</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
@@ -1377,7 +1329,7 @@
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>476,2 TL</t>
+          <t>666,67 TL</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
@@ -1429,7 +1381,7 @@
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>428,58 TL</t>
+          <t>571,43 TL</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-08 12:55:28 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -736,12 +732,24 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 99,71 TL</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr"/>
-      <c r="I6" s="14" t="inlineStr"/>
-      <c r="J6" s="14" t="inlineStr"/>
+          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -803,11 +811,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -823,11 +827,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -843,11 +843,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -863,11 +859,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -892,15 +884,15 @@
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -914,13 +906,29 @@
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 57,5 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr"/>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -934,21 +942,29 @@
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr"/>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-09 12:41:48 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -732,7 +736,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
+          <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -750,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -811,7 +811,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -827,7 +831,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -843,7 +851,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -859,7 +871,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -881,18 +897,22 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -905,12 +925,12 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 57,5 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -918,17 +938,13 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="J13" s="14" t="inlineStr"/>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -941,30 +957,30 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-10 12:00:42 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -930,7 +938,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -938,13 +950,21 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -962,8 +982,16 @@
           <t>3.500 TL - 13.500 TL</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
@@ -980,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-11 12:12:57 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -901,11 +901,7 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -933,11 +929,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -977,11 +969,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-12 14:34:49 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -901,7 +901,11 @@
           <t>WU: 1.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -929,7 +933,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -947,11 +955,7 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
+      <c r="J13" s="14" t="inlineStr"/>
       <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
@@ -969,7 +973,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -991,11 +999,7 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>
@@ -1384,11 +1388,7 @@
           <t>666,67 TL</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>780 TL</t>
-        </is>
-      </c>
+      <c r="E24" s="14" t="inlineStr"/>
       <c r="F24" s="14" t="inlineStr">
         <is>
           <t>600 TL</t>
@@ -1436,11 +1436,7 @@
           <t>571,43 TL</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>780 TL</t>
-        </is>
-      </c>
+      <c r="E25" s="14" t="inlineStr"/>
       <c r="F25" s="14" t="inlineStr">
         <is>
           <t>600 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-13 13:41:00 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -728,11 +728,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -744,21 +740,9 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="I6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -898,14 +882,10 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -916,11 +896,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -933,16 +909,8 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
       <c r="H13" s="14" t="inlineStr">
@@ -950,17 +918,9 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr"/>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -973,16 +933,8 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2.170 TL - 2.170 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
+      <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>2.785,72 TL - 12.380,95 TL</t>
@@ -1000,11 +952,7 @@
       </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr"/>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -1388,7 +1336,11 @@
           <t>666,67 TL</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr"/>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>780 TL</t>
+        </is>
+      </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
           <t>600 TL</t>
@@ -1436,7 +1388,11 @@
           <t>571,43 TL</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr"/>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>780 TL</t>
+        </is>
+      </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
           <t>600 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-14 11:19:07 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,16 +718,8 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
@@ -742,7 +734,11 @@
       </c>
       <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr"/>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -880,11 +876,7 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
@@ -896,7 +888,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -904,23 +900,19 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
+      <c r="C13" s="14" t="inlineStr"/>
       <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr"/>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr"/>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 69,62 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -928,31 +920,23 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40.000 TL - 2.485,72 TL</t>
-        </is>
-      </c>
+      <c r="C14" s="14" t="inlineStr"/>
       <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr"/>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-15 10:57:32 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -718,9 +718,21 @@
           <t>DÜZENLİ EFT</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr"/>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -732,8 +744,16 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -876,8 +896,16 @@
           <t>GİDEN SWIFT</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -900,17 +928,41 @@
           <t>GELEN SWIFT</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+        </is>
+      </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
-      <c r="I13" s="14" t="inlineStr"/>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 69,62 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
         </is>
       </c>
     </row>
@@ -920,18 +972,42 @@
           <t>GİDEN SWIFT - Mobil</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr"/>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>40.000 TL - 2.485,72 TL</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>2.170 TL - 2.170 TL</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
           <t>1.196,51 TL - 5.583,74 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-16 10:49:09 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,11 +601,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>35,71 TL - 35,71 TL</t>
-        </is>
-      </c>
+      <c r="C2" s="14" t="inlineStr"/>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -898,7 +894,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
+          <t>WU: 3.000,01 USD–</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -930,7 +926,7 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -940,16 +936,12 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 57,5 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -997,11 +989,7 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-17 10:14:34 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -601,7 +601,11 @@
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr"/>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>35,71 TL - 35,71 TL</t>
+        </is>
+      </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
           <t>33,33 TL - 33,33 TL</t>
@@ -732,7 +736,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 99,71 TL</t>
+          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -811,11 +815,7 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
-        </is>
-      </c>
+      <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -831,11 +831,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
-        </is>
-      </c>
+      <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -851,11 +847,7 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -871,11 +863,7 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
-        </is>
-      </c>
+      <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -894,7 +882,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 3.000,01 USD–</t>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -904,11 +892,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
-        </is>
-      </c>
+      <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -926,7 +910,7 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 3.295,24 TL</t>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -936,12 +920,16 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 57,5 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -954,7 +942,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 69,62 TL</t>
         </is>
       </c>
     </row>
@@ -984,12 +972,12 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
-        <is>
-          <t>8.300 TL - 7,97 TL</t>
-        </is>
-      </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-18 10:30:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -736,7 +732,7 @@
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>8.300,01 TL - 57,5 TL - 115 TL</t>
+          <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -815,7 +811,11 @@
       <c r="D8" s="14" t="inlineStr"/>
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>19,94 TRY - 39,88 TRY - 398,84 TRY</t>
+        </is>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
@@ -831,7 +831,11 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>13,92 TRY - 27,85 TRY - 199,42 TRY</t>
+        </is>
+      </c>
       <c r="H9" s="14" t="inlineStr"/>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
@@ -847,7 +851,11 @@
       <c r="D10" s="14" t="inlineStr"/>
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H10" s="14" t="inlineStr"/>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
@@ -863,7 +871,11 @@
       <c r="D11" s="14" t="inlineStr"/>
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TRY - 7,98 TRY - 99,71 TRY</t>
+        </is>
+      </c>
       <c r="H11" s="14" t="inlineStr"/>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
@@ -885,14 +897,14 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Şube (Kasadan): %0,5; Şube (Hesaptan): %0,75; İnternet: 15 USD</t>
+        </is>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
@@ -913,11 +925,7 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -942,7 +950,7 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 69,62 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
         </is>
       </c>
     </row>
@@ -957,11 +965,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -972,7 +976,11 @@
           <t>2.785,72 TL - 12.380,95 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>8.300 TL - 7,97 TL</t>
+        </is>
+      </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
           <t>3.000 TL - 6.000 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-19 12:17:47 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-20 11:00:37 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,11 +754,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -898,10 +894,14 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 3.000,01 USD–9,51 USD</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr"/>
+          <t>WU: 1.000,01 USD–9,51 USD</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -912,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -929,7 +925,11 @@
           <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -947,16 +947,8 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="J13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -969,7 +961,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -991,16 +987,8 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-21 11:17:51 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -754,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -894,7 +898,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>WU: 1.000,01 USD–9,51 USD</t>
+          <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -932,7 +936,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -947,7 +951,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
       <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
@@ -987,7 +995,11 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
       <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-22 11:16:17 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -916,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -936,7 +940,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 1 TL | Azami 11.380 TL</t>
+          <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr"/>
@@ -956,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1000,7 +1008,11 @@
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-23 11:07:49 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,11 +723,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="D6" s="14" t="inlineStr"/>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -901,11 +897,7 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
-        </is>
-      </c>
+      <c r="D12" s="14" t="inlineStr"/>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -930,14 +922,10 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
-        </is>
-      </c>
+          <t>Hesaba: Asgari 0 TL | Azami 9.999.999.999.999 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -977,11 +965,7 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>3.500 TL - 13.500 TL</t>
-        </is>
-      </c>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-24 10:23:34 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -723,7 +723,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -897,7 +901,11 @@
           <t>WU: 3.000,01 USD–9,51 USD</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>WU: 6 USD–12 USD; Diğer: 700 TL–4.000 TL</t>
+        </is>
+      </c>
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr">
@@ -922,10 +930,14 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Hesaba: Asgari 0 TL | Azami 9.999.999.999.999 TL</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr"/>
+          <t>Hesaba: Asgari 0 TL | Azami 0,94 TL</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.190 TL</t>
+        </is>
+      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.114 TL</t>
@@ -933,16 +945,8 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr"/>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -965,7 +969,11 @@
           <t>40.000 TL - 2.485,72 TL</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>3.500 TL - 13.500 TL</t>
+        </is>
+      </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
           <t>2.170 TL - 2.170 TL</t>
@@ -981,11 +989,7 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-25 10:51:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -945,8 +945,16 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
-      <c r="I13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
@@ -989,7 +997,11 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-26 12:22:09 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -987,11 +987,7 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>2.785,72 TL - 12.380,95 TL</t>
-        </is>
-      </c>
+      <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>

</xml_diff>

<commit_message>
Update benchmark: 2026-10-27 11:42:07 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -739,26 +739,18 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="J6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="K6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -916,11 +908,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -945,26 +933,18 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
-        </is>
-      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -987,28 +967,24 @@
           <t>2.170 TL - 2.170 TL</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2.785,72 TL - 12.380,95 TL</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>3.000 TL - 6.000 TL</t>
-        </is>
-      </c>
+      <c r="H14" s="14" t="inlineStr"/>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-28 12:14:00 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -739,7 +739,11 @@
           <t>8.300,01 TL - 99,71 TL</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
           <t>8.300,01 TL - 199,41 TL</t>
@@ -750,7 +754,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>7,97 TL - 15,96 TL - 199,41 TL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -908,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -933,7 +945,11 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
+        </is>
+      </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
@@ -944,7 +960,11 @@
           <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -977,14 +997,22 @@
           <t>8.300 TL - 7,97 TL</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>3.000 TL - 6.000 TL</t>
+        </is>
+      </c>
       <c r="I14" s="14" t="inlineStr"/>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>1.554,97 TL - 7.784 TL</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-30 12:14:41 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -749,11 +749,7 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>8.300,01 TL - 199,41 TL</t>
-        </is>
-      </c>
+      <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -916,11 +912,7 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
-        </is>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -955,16 +947,8 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
-        </is>
-      </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
-        </is>
-      </c>
+      <c r="J13" s="14" t="inlineStr"/>
+      <c r="K13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1003,16 +987,8 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>1.554,97 TL - 7.784 TL</t>
-        </is>
-      </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>1.196,51 TL - 5.583,74 TL</t>
-        </is>
-      </c>
+      <c r="J14" s="14" t="inlineStr"/>
+      <c r="K14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Update benchmark: 2026-10-31 11:47:21 UTC
</commit_message>
<xml_diff>
--- a/docs/Benchmark_Results.xlsx
+++ b/docs/Benchmark_Results.xlsx
@@ -749,7 +749,11 @@
           <t>8.300,01 TL - 199,41 TL</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>8.300,01 TL - 199,41 TL</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
           <t>7,97 TL - 15,96 TL - 199,41 TL</t>
@@ -912,7 +916,11 @@
       <c r="H12" s="14" t="inlineStr"/>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
-      <c r="K12" s="14" t="inlineStr"/>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>WU: ,USD–; Diğer: 529 TL–4.454,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -947,8 +955,16 @@
           <t>Hesaba: Asgari 1 TL | Azami 7,97 TL</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr"/>
-      <c r="K13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.303 TL</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Hesaba: Asgari 1 TL | Azami 1.133 TL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -987,8 +1003,16 @@
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr"/>
-      <c r="J14" s="14" t="inlineStr"/>
-      <c r="K14" s="14" t="inlineStr"/>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>1.554,97 TL - 7.784 TL</t>
+        </is>
+      </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>1.196,51 TL - 5.583,74 TL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">

</xml_diff>